<commit_message>
Fix idiom 行不由徑 (was mistyped as 不行由徑)
Correct the idiom, reorder its zhuyin to match, and fix the same
typo in the example sentence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/成語.xlsx
+++ b/docs/成語.xlsx
@@ -2595,16 +2595,16 @@
         <v>德性篇</v>
       </c>
       <c r="B133" t="str">
-        <v>不行由徑</v>
+        <v>行不由徑</v>
       </c>
       <c r="C133" t="str">
-        <v>ㄅㄨˋ ㄒㄧㄥˊ ㄧㄡˊ ㄐㄧㄥˋ</v>
+        <v>ㄒㄧㄥˊ ㄅㄨˋ ㄧㄡˊ ㄐㄧㄥˋ</v>
       </c>
       <c r="D133" t="str">
         <v>走路不走捷徑。比喻行事光明正大，不投機取巧。</v>
       </c>
       <c r="E133" t="str">
-        <v>他做生意講求誠信，一向不行由徑，因此獲得客戶的長久信任。</v>
+        <v>他做生意講求誠信，一向行不由徑，因此獲得客戶的長久信任。</v>
       </c>
     </row>
     <row r="134">

</xml_diff>